<commit_message>
all status print done
</commit_message>
<xml_diff>
--- a/workStatus/workStatus.xlsx
+++ b/workStatus/workStatus.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="59">
   <si>
     <t>s/n</t>
   </si>
@@ -106,9 +106,6 @@
     <t>Dispactch list , delivery, Edit</t>
   </si>
   <si>
-    <t>excel dispath list,  copy, coplete</t>
-  </si>
-  <si>
     <t>Delivery Invoice</t>
   </si>
   <si>
@@ -121,15 +118,9 @@
     <t>cancel</t>
   </si>
   <si>
-    <t>Print edit</t>
-  </si>
-  <si>
     <t>All status</t>
   </si>
   <si>
-    <t>Pint Edit</t>
-  </si>
-  <si>
     <t>Send percel</t>
   </si>
   <si>
@@ -187,10 +178,19 @@
     <t>Searchng, List and details</t>
   </si>
   <si>
-    <t>working on Print</t>
-  </si>
-  <si>
     <t>Edit Details  Requried</t>
+  </si>
+  <si>
+    <t>List, Print  edit</t>
+  </si>
+  <si>
+    <t>List, Print Edit</t>
+  </si>
+  <si>
+    <t>Edit Detail Info Requred</t>
+  </si>
+  <si>
+    <t>excel dispath list,  copy, complete</t>
   </si>
 </sst>
 </file>
@@ -607,7 +607,7 @@
     <col min="5" max="5" width="50.7109375" customWidth="1"/>
     <col min="6" max="6" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:9" x14ac:dyDescent="0.25">
@@ -789,7 +789,7 @@
         <v>27</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="F12" s="3" t="s">
         <v>8</v>
@@ -815,7 +815,7 @@
         <v>8</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
@@ -826,17 +826,17 @@
         <v>17</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>30</v>
+        <v>58</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="G14" s="6"/>
       <c r="H14" s="6" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="I14" s="2"/>
     </row>
@@ -846,10 +846,10 @@
         <v>17</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>8</v>
@@ -864,58 +864,62 @@
         <v>18</v>
       </c>
       <c r="D16" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E16" s="2" t="s">
-        <v>33</v>
-      </c>
       <c r="F16" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B17" s="2"/>
-      <c r="C17" s="2">
+      <c r="C17" s="3">
         <v>18</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F17" s="2" t="s">
+      <c r="D17" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="F17" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G17" s="2" t="s">
-        <v>57</v>
+      <c r="G17" s="3" t="s">
+        <v>14</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="I17" s="2"/>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B18" s="2"/>
-      <c r="C18" s="2">
+      <c r="C18" s="3">
         <v>19</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
+      <c r="D18" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>57</v>
+      </c>
       <c r="I18" s="2"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.25">
@@ -924,10 +928,10 @@
         <v>20</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>8</v>
@@ -942,15 +946,15 @@
         <v>21</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="I20" s="2"/>
     </row>
@@ -960,10 +964,10 @@
         <v>22</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>8</v>
@@ -978,10 +982,10 @@
         <v>23</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>8</v>
@@ -996,10 +1000,10 @@
         <v>23</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F23" s="3" t="s">
         <v>8</v>
@@ -1014,10 +1018,10 @@
         <v>24</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F24" s="3" t="s">
         <v>8</v>
@@ -1032,10 +1036,10 @@
         <v>24</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>8</v>

</xml_diff>

<commit_message>
excel dispatch copy option pending
</commit_message>
<xml_diff>
--- a/workStatus/workStatus.xlsx
+++ b/workStatus/workStatus.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="60">
   <si>
     <t>s/n</t>
   </si>
@@ -191,13 +191,16 @@
   </si>
   <si>
     <t>excel dispath list,  copy, complete</t>
+  </si>
+  <si>
+    <t>details required (Copy pending)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -214,20 +217,13 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -237,11 +233,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -269,12 +260,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -285,19 +275,15 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="2">
     <cellStyle name="Good" xfId="1" builtinId="26"/>
-    <cellStyle name="Neutral" xfId="2" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -356,7 +342,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -391,7 +377,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -821,22 +807,22 @@
       <c r="I13" s="2"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B14" s="2"/>
-      <c r="C14" s="6">
+      <c r="B14" s="3"/>
+      <c r="C14" s="3">
         <v>17</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D14" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="E14" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="F14" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6" t="s">
-        <v>41</v>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3" t="s">
+        <v>59</v>
       </c>
       <c r="I14" s="2"/>
     </row>

</xml_diff>

<commit_message>
delivery and added reject
</commit_message>
<xml_diff>
--- a/workStatus/workStatus.xlsx
+++ b/workStatus/workStatus.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="59">
   <si>
     <t>s/n</t>
   </si>
@@ -161,9 +161,6 @@
   </si>
   <si>
     <t>Process order list, print, Edit and cancel</t>
-  </si>
-  <si>
-    <t>working on Edit</t>
   </si>
   <si>
     <t>excel dispath</t>
@@ -788,22 +785,22 @@
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B13" s="2"/>
-      <c r="C13" s="2">
+      <c r="C13" s="3">
         <v>16</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D13" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="E13" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F13" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="H13" s="2"/>
+      <c r="F13" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H13" s="3"/>
       <c r="I13" s="2"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.25">
@@ -812,17 +809,17 @@
         <v>17</v>
       </c>
       <c r="D14" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="F14" s="3" t="s">
         <v>50</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>51</v>
       </c>
       <c r="G14" s="3"/>
       <c r="H14" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I14" s="2"/>
     </row>
@@ -835,7 +832,7 @@
         <v>30</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>8</v>
@@ -846,22 +843,22 @@
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B16" s="2"/>
-      <c r="C16" s="2">
+      <c r="C16" s="3">
         <v>18</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D16" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="E16" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="F16" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="G16" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="G16" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="H16" s="2"/>
+      <c r="H16" s="3"/>
       <c r="I16" s="2"/>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.25">
@@ -873,7 +870,7 @@
         <v>33</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F17" s="3" t="s">
         <v>11</v>
@@ -882,7 +879,7 @@
         <v>14</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I17" s="2"/>
     </row>
@@ -895,7 +892,7 @@
         <v>34</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F18" s="3" t="s">
         <v>11</v>
@@ -904,7 +901,7 @@
         <v>14</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="I18" s="2"/>
     </row>

</xml_diff>

<commit_message>
stock list edit delete done
</commit_message>
<xml_diff>
--- a/workStatus/workStatus.xlsx
+++ b/workStatus/workStatus.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
@@ -339,7 +339,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -374,7 +374,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -727,20 +727,20 @@
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B10" s="2"/>
-      <c r="C10" s="2">
+      <c r="C10" s="3">
         <v>13</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F10" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
+      <c r="F10" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
       <c r="I10" s="2"/>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.25">

</xml_diff>